<commit_message>
Change content - 07042026
</commit_message>
<xml_diff>
--- a/DA24TTC-To1-220236.xlsx
+++ b/DA24TTC-To1-220236.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="137">
   <si>
     <t>Đại học Trà Vinh</t>
   </si>
@@ -409,9 +409,6 @@
     <t>Trường</t>
   </si>
   <si>
-    <t>Buổi thuc hanh 1</t>
-  </si>
-  <si>
     <t>Bài 1</t>
   </si>
   <si>
@@ -422,6 +419,14 @@
   </si>
   <si>
     <t>Không có học lý thuyết</t>
+  </si>
+  <si>
+    <t>Buổi thực hành 2
+Định dạng CSS cho trang thông tin cá nhân</t>
+  </si>
+  <si>
+    <t>Buổi thuc hanh 1
+Tạo trang thông tin cá nhân và công bố Github Pages</t>
   </si>
 </sst>
 </file>
@@ -561,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -575,7 +580,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -597,6 +601,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -947,43 +955,43 @@
     <col min="9" max="9" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="G1" s="5" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="G1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="5"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="G2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D4" s="5" t="s">
+      <c r="H2" s="14"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D4" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D5" s="5" t="s">
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D5" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -997,7 +1005,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -1011,7 +1019,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>14</v>
       </c>
@@ -1025,7 +1033,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="142.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -1045,19 +1053,22 @@
         <v>23</v>
       </c>
       <c r="G11" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="J11" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="J11" s="8" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
@@ -1078,10 +1089,10 @@
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I12" s="6"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>30</v>
       </c>
@@ -1102,10 +1113,10 @@
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I13" s="6"/>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
@@ -1126,10 +1137,10 @@
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I14" s="6"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>37</v>
       </c>
@@ -1150,10 +1161,10 @@
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I15" s="6"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>41</v>
       </c>
@@ -1174,8 +1185,8 @@
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="9"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
@@ -1198,8 +1209,8 @@
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="9"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -1222,8 +1233,8 @@
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="9"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
@@ -1246,8 +1257,8 @@
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="9"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -1270,8 +1281,8 @@
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="9"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="8"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -1294,8 +1305,8 @@
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="9"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="8"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
@@ -1320,8 +1331,8 @@
         <v>4</v>
       </c>
       <c r="H22" s="3"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="9"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
@@ -1344,8 +1355,8 @@
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="9"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="8"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -1368,8 +1379,8 @@
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="9"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -1392,8 +1403,8 @@
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="9"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="8"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
@@ -1416,8 +1427,8 @@
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="9"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="8"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -1440,8 +1451,8 @@
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="9"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="8"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
@@ -1464,8 +1475,8 @@
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="9"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="8"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
@@ -1488,8 +1499,8 @@
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="9"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="8"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
@@ -1512,8 +1523,8 @@
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="9"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="8"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
@@ -1536,8 +1547,8 @@
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="9"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="8"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
@@ -1560,8 +1571,8 @@
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="9"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="8"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
@@ -1584,8 +1595,8 @@
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="9"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="8"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
@@ -1608,8 +1619,8 @@
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="9"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="8"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
@@ -1632,8 +1643,8 @@
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="9"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="8"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
@@ -1656,8 +1667,8 @@
       </c>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="9"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="8"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
@@ -1680,36 +1691,36 @@
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="9"/>
-    </row>
-    <row r="38" spans="1:10" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+      <c r="I37" s="6"/>
+      <c r="J37" s="8"/>
+    </row>
+    <row r="38" spans="1:10" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="F38" s="11" t="s">
+      <c r="F38" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="G38" s="10">
+      <c r="G38" s="9">
         <v>4</v>
       </c>
-      <c r="H38" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="I38" s="12"/>
-      <c r="J38" s="13"/>
+      <c r="H38" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="I38" s="11"/>
+      <c r="J38" s="12"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
@@ -1732,8 +1743,8 @@
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
-      <c r="I39" s="7"/>
-      <c r="J39" s="9"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>